<commit_message>
additions to matching diagram python script with ISA calculator
</commit_message>
<xml_diff>
--- a/wing_initial_planform.xlsx
+++ b/wing_initial_planform.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adria\Desktop\TU Delft\AE 26-27\(AE2111-I) Aerospace System Design\Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB71E16-B9C8-4638-BA14-B52A3F1C88A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3C198B-FE9E-433A-A763-00D4E4D2953C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1464" yWindow="1464" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>Parameter</t>
   </si>
@@ -96,18 +107,12 @@
     <t>Landing distance</t>
   </si>
   <si>
-    <t>Leading Edge Mean Aerodynamic Cord (fr*nch mcdonalds)</t>
-  </si>
-  <si>
     <t>Lift-to-drag cruise</t>
   </si>
   <si>
     <t>MAC</t>
   </si>
   <si>
-    <t xml:space="preserve">Mach number cruise </t>
-  </si>
-  <si>
     <t>Maximum payload</t>
   </si>
   <si>
@@ -184,6 +189,24 @@
   </si>
   <si>
     <t>Cruise altitude IN METERS</t>
+  </si>
+  <si>
+    <t>Mass fraction take-off</t>
+  </si>
+  <si>
+    <t>Mass fraction cruise</t>
+  </si>
+  <si>
+    <t>Mass fraction landing</t>
+  </si>
+  <si>
+    <t>Leading Edge MAC</t>
+  </si>
+  <si>
+    <t>Mach number cruise</t>
+  </si>
+  <si>
+    <t>Number of engines</t>
   </si>
 </sst>
 </file>
@@ -502,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49.109375" bestFit="1" customWidth="1"/>
@@ -574,7 +597,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B9">
         <v>12496.8</v>
@@ -686,7 +709,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="B23">
         <v>0.80104231299999995</v>
@@ -694,7 +717,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24">
         <v>15.99244976</v>
@@ -702,7 +725,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25">
         <v>1.9837065780000001</v>
@@ -710,7 +733,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="B26">
         <v>0.68</v>
@@ -718,205 +741,238 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B27">
-        <v>1010</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="B28">
-        <v>12260.26592</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="B29">
-        <v>7478.7622099999999</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B30">
-        <v>0.61</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B31">
-        <v>0.81221284400000004</v>
+        <v>12260.26592</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="B32">
-        <v>7.4999999999999997E-3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B33">
-        <v>0.97</v>
+        <v>7478.7622099999999</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B34">
-        <v>2.7131115100000001</v>
+        <v>0.61</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B35">
-        <v>3.3174846150000001</v>
+        <v>0.81221284400000004</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B36">
-        <v>295.04231900000002</v>
+        <v>7.4999999999999997E-3</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B37">
-        <v>48.780487800000003</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B38">
-        <v>13.57484339</v>
+        <v>2.7131115100000001</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B39">
-        <v>10.5639649</v>
+        <v>3.3174846150000001</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B40">
-        <v>1250</v>
+        <v>295.04231900000002</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B41">
-        <v>1250</v>
+        <v>48.780487800000003</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B42">
-        <v>0.36312480600000002</v>
+        <v>13.57484339</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B43">
-        <v>216.65</v>
+        <v>10.5639649</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B44">
-        <v>0.42499999999999999</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B45">
-        <v>0.985198091</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B46">
-        <v>51098.658130000003</v>
+        <v>0.36312480600000002</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B47">
-        <v>15.913062549999999</v>
+        <v>216.65</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B48">
-        <v>29.064674539999999</v>
+        <v>0.42499999999999999</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B49">
-        <v>4136.7102400000003</v>
+        <v>0.985198091</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B50">
-        <v>15.7178158</v>
+        <v>51098.658130000003</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B51">
+        <v>15.913062549999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>46</v>
+      </c>
+      <c r="B52">
+        <v>29.064674539999999</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>47</v>
+      </c>
+      <c r="B53">
+        <v>4136.7102400000003</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>48</v>
+      </c>
+      <c r="B54">
+        <v>15.7178158</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>49</v>
+      </c>
+      <c r="B55">
         <v>2.12E-2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added necessary hinge line calculations for flap.py
</commit_message>
<xml_diff>
--- a/wing_initial_planform.xlsx
+++ b/wing_initial_planform.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adria\Desktop\TU Delft\AE 26-27\(AE2111-I) Aerospace System Design\Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3C198B-FE9E-433A-A763-00D4E4D2953C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95974E32-CC09-4E5C-B8D7-38C1B0428EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1464" yWindow="1464" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -568,7 +568,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
edited planform excel and added drag polar script
</commit_message>
<xml_diff>
--- a/wing_initial_planform.xlsx
+++ b/wing_initial_planform.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adria\Desktop\TU Delft\AE 26-27\(AE2111-I) Aerospace System Design\Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{713D42C3-B1D6-4772-9F26-4D02BE1D4AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A99C83-33F7-4A8C-B5EE-8EDF43EA36BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>Parameter</t>
   </si>
@@ -199,6 +199,15 @@
   </si>
   <si>
     <t>Wing span</t>
+  </si>
+  <si>
+    <t>CL alpha flapped</t>
+  </si>
+  <si>
+    <t>a0L landing</t>
+  </si>
+  <si>
+    <t>a0L take-off</t>
   </si>
 </sst>
 </file>
@@ -244,10 +253,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -918,9 +928,30 @@
         <v>5.519474327833759</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B57">
+        <v>0.14938077070380501</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B58">
+        <v>-10.2511706715958</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B59">
+        <v>-7.8507804477305303</v>
+      </c>
+    </row>
     <row r="60" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="61" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="62" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Updated aileron.py and excel
</commit_message>
<xml_diff>
--- a/wing_initial_planform.xlsx
+++ b/wing_initial_planform.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adria\Desktop\TU Delft\AE 26-27\(AE2111-I) Aerospace System Design\Code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jedrzej\Documents\Python\system_design\B09\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A99C83-33F7-4A8C-B5EE-8EDF43EA36BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8805BF90-AF64-4A36-83D8-632D5EF8EF66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="kHHFuU2Gy+4Gka7AgTnrw+aeKvwWd4PTC7Y6sbZGr1E="/>
@@ -253,11 +253,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -929,15 +928,15 @@
       </c>
     </row>
     <row r="57" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="3" t="s">
+      <c r="A57" t="s">
         <v>58</v>
       </c>
       <c r="B57">
-        <v>0.14938077070380501</v>
+        <v>8.5588877017395184</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="3" t="s">
+      <c r="A58" t="s">
         <v>59</v>
       </c>
       <c r="B58">
@@ -945,7 +944,7 @@
       </c>
     </row>
     <row r="59" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="3" t="s">
+      <c r="A59" t="s">
         <v>60</v>
       </c>
       <c r="B59">

</xml_diff>

<commit_message>
changes to flap and ISA correction, and sharpness/CL_alpha calculations
</commit_message>
<xml_diff>
--- a/wing_initial_planform.xlsx
+++ b/wing_initial_planform.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adria\Desktop\TU Delft\AE 26-27\(AE2111-I) Aerospace System Design\Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A99C83-33F7-4A8C-B5EE-8EDF43EA36BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B114D841-2383-4791-A87C-52F48088885E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1812" yWindow="1812" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>Parameter</t>
   </si>
@@ -208,6 +208,9 @@
   </si>
   <si>
     <t>a0L take-off</t>
+  </si>
+  <si>
+    <t>CD0</t>
   </si>
 </sst>
 </file>
@@ -253,11 +256,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -929,7 +931,7 @@
       </c>
     </row>
     <row r="57" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="3" t="s">
+      <c r="A57" t="s">
         <v>58</v>
       </c>
       <c r="B57">
@@ -937,7 +939,7 @@
       </c>
     </row>
     <row r="58" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="3" t="s">
+      <c r="A58" t="s">
         <v>59</v>
       </c>
       <c r="B58">
@@ -945,14 +947,21 @@
       </c>
     </row>
     <row r="59" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="3" t="s">
+      <c r="A59" t="s">
         <v>60</v>
       </c>
       <c r="B59">
         <v>-7.8507804477305303</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>61</v>
+      </c>
+      <c r="B60">
+        <v>2.12E-2</v>
+      </c>
+    </row>
     <row r="61" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="62" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="63" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>